<commit_message>
feat: GasAgas v2.1 - Multi-role workers + NuevaRecepcion fixes + UI improvements
</commit_message>
<xml_diff>
--- a/replicacion_control_envases.xlsx
+++ b/replicacion_control_envases.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Manuel Gonzalez\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\proyectos\Gases_agas\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,6 +14,9 @@
   <sheets>
     <sheet name="recepcion" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">recepcion!$A$1:$P$36</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -216,9 +219,6 @@
   </cellStyleXfs>
   <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -236,9 +236,6 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -253,12 +250,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -266,6 +257,18 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -612,489 +615,495 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A2:P36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="10" width="4.7109375" style="2" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5703125" style="10" customWidth="1"/>
-    <col min="13" max="14" width="8.7109375" style="10" customWidth="1"/>
-    <col min="15" max="15" width="16" style="2" customWidth="1"/>
-    <col min="16" max="16" width="32.42578125" style="2" customWidth="1"/>
-    <col min="17" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="10" width="4.7109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" style="8" customWidth="1"/>
+    <col min="13" max="14" width="8.7109375" style="8" customWidth="1"/>
+    <col min="15" max="15" width="16" style="1" customWidth="1"/>
+    <col min="16" max="16" width="32.42578125" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:16" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="O2" s="21" t="s">
+      <c r="O2" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="P2" s="12">
+      <c r="P2" s="10">
         <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="18" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-      <c r="M4" s="9"/>
-      <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="9"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
     </row>
     <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.2">
-      <c r="O6" s="3" t="s">
+      <c r="O6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="P6" s="4">
+      <c r="P6" s="3">
         <v>46254</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="17"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="17"/>
-      <c r="H8" s="17"/>
-      <c r="I8" s="17"/>
-      <c r="J8" s="17"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="10" t="s">
+      <c r="C8" s="18"/>
+      <c r="D8" s="18"/>
+      <c r="E8" s="18"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="18"/>
+      <c r="M8" s="18"/>
+      <c r="N8" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="O8" s="17"/>
-      <c r="P8" s="17"/>
+      <c r="O8" s="18"/>
+      <c r="P8" s="18"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="1" t="s">
+      <c r="D10" s="18"/>
+      <c r="E10" s="18"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="18"/>
+      <c r="M10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="N10" s="1"/>
-      <c r="O10" s="17"/>
-      <c r="P10" s="17"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="18"/>
+      <c r="P10" s="18"/>
     </row>
     <row r="12" spans="1:16" ht="64.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G12" s="5" t="s">
+      <c r="G12" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-      <c r="K12" s="6" t="s">
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L12" s="7" t="s">
+      <c r="L12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="M12" s="6" t="s">
+      <c r="M12" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="N12" s="6" t="s">
+      <c r="N12" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="O12" s="7" t="s">
+      <c r="O12" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="P12" s="6" t="s">
+      <c r="P12" s="5" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
+      <c r="J13" s="7"/>
+      <c r="K13" s="7"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="7"/>
+      <c r="P13" s="7"/>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
+      <c r="J14" s="7"/>
+      <c r="K14" s="7"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="7"/>
+      <c r="P14" s="7"/>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
+      <c r="J15" s="7"/>
+      <c r="K15" s="7"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="7"/>
+      <c r="P15" s="7"/>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="8"/>
-      <c r="P16" s="8"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
+      <c r="J16" s="7"/>
+      <c r="K16" s="7"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="7"/>
+      <c r="P16" s="7"/>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="8"/>
-      <c r="P17" s="8"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
+      <c r="J17" s="7"/>
+      <c r="K17" s="7"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="7"/>
+      <c r="P17" s="7"/>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
-      <c r="I18" s="8"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="8"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+      <c r="I18" s="7"/>
+      <c r="J18" s="7"/>
+      <c r="K18" s="7"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="7"/>
+      <c r="P18" s="7"/>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="8"/>
-      <c r="P19" s="8"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
+      <c r="J19" s="7"/>
+      <c r="K19" s="7"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="7"/>
+      <c r="P19" s="7"/>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="8"/>
-      <c r="P20" s="8"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
+      <c r="J20" s="7"/>
+      <c r="K20" s="7"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="7"/>
+      <c r="P20" s="7"/>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="8"/>
-      <c r="P21" s="8"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
+      <c r="J21" s="7"/>
+      <c r="K21" s="7"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="7"/>
+      <c r="P21" s="7"/>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="11"/>
-      <c r="M22" s="11"/>
-      <c r="N22" s="11"/>
-      <c r="O22" s="8"/>
-      <c r="P22" s="8"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7"/>
+      <c r="K22" s="7"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="7"/>
+      <c r="P22" s="7"/>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="11"/>
-      <c r="M23" s="11"/>
-      <c r="N23" s="11"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="8"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7"/>
+      <c r="K23" s="7"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+      <c r="O23" s="7"/>
+      <c r="P23" s="7"/>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="8"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="11"/>
-      <c r="M24" s="11"/>
-      <c r="N24" s="11"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="8"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
+      <c r="J24" s="7"/>
+      <c r="K24" s="7"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+      <c r="O24" s="7"/>
+      <c r="P24" s="7"/>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="8"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
+      <c r="J25" s="7"/>
+      <c r="K25" s="7"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="7"/>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="8"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="11"/>
-      <c r="M26" s="11"/>
-      <c r="N26" s="11"/>
-      <c r="O26" s="8"/>
-      <c r="P26" s="8"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7"/>
+      <c r="K26" s="7"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="7"/>
+      <c r="P26" s="7"/>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A27" s="13"/>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="13"/>
-      <c r="H27" s="13"/>
-      <c r="I27" s="13"/>
-      <c r="J27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
-      <c r="O27" s="13"/>
-      <c r="P27" s="13"/>
+      <c r="A27" s="11"/>
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="11"/>
+      <c r="P27" s="11"/>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A28" s="13"/>
-      <c r="B28" s="13"/>
-      <c r="C28" s="13"/>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="13"/>
-      <c r="G28" s="13"/>
-      <c r="H28" s="13"/>
-      <c r="I28" s="13"/>
-      <c r="J28" s="13"/>
-      <c r="K28" s="13"/>
-      <c r="L28" s="14"/>
-      <c r="M28" s="14"/>
-      <c r="N28" s="14"/>
-      <c r="O28" s="13"/>
-      <c r="P28" s="13"/>
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="11"/>
+      <c r="P28" s="11"/>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
-      <c r="J30" s="17"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17"/>
-      <c r="M30" s="17"/>
-      <c r="O30" s="2" t="s">
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="18"/>
+      <c r="M30" s="18"/>
+      <c r="O30" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="P30" s="18"/>
+      <c r="P30" s="14"/>
     </row>
     <row r="31" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="32" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A32" s="15" t="s">
+      <c r="A32" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="17"/>
-      <c r="F32" s="17"/>
-      <c r="G32" s="17"/>
-      <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
-      <c r="J32" s="17"/>
-      <c r="K32" s="16" t="s">
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="L32" s="16"/>
-      <c r="M32" s="17"/>
-      <c r="N32" s="17"/>
-      <c r="O32" s="2" t="s">
+      <c r="L32" s="20"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+      <c r="O32" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="P32" s="18"/>
+      <c r="P32" s="14"/>
     </row>
     <row r="33" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A34" s="20" t="s">
+      <c r="A34" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="O34" s="2" t="s">
+      <c r="O34" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="P34" s="19"/>
+      <c r="P34" s="15"/>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A35" s="20" t="s">
+      <c r="A35" s="16" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A36" s="20" t="s">
+      <c r="A36" s="16" t="s">
         <v>27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A4:P4"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="C8:M8"/>
     <mergeCell ref="D10:L10"/>
     <mergeCell ref="O10:P10"/>
     <mergeCell ref="M10:N10"/>
@@ -1102,12 +1111,10 @@
     <mergeCell ref="K32:L32"/>
     <mergeCell ref="M32:N32"/>
     <mergeCell ref="E30:M30"/>
-    <mergeCell ref="A4:P4"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="C8:M8"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.15748031496062992" right="0.15748031496062992" top="0.39370078740157483" bottom="0.39370078740157483" header="0.51181102362204722" footer="0.51181102362204722"/>
+  <pageSetup scale="97" fitToWidth="0" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>